<commit_message>
feat(006): convergência da fase C (T157: programação × geração no nível do conjunto; G5 nas legendas de programação), portão da fase C (T116) e referências da UFV Seriemas 1 e da EOL Praia Formosa
</commit_message>
<xml_diff>
--- a/reports/seriemas_1/perfil_estatistico_anual.xlsx
+++ b/reports/seriemas_1/perfil_estatistico_anual.xlsx
@@ -16,21 +16,24 @@
     <sheet name="OMITIDOS" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="CONF_NAO_APLICAVEIS" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="PARAMETROS" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="REN_FC_ANUAL" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="REN_FC_MENSAL" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="REN_CORTE_ANUAL" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="REN_CORTE_MENSAL" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="REN_CORTE_RAZAO" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="REN_RECURSO_FAIXAS" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="CONF_G1_PARES" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="CONF_G1_MENSAL" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="CONF_G2_MENSAL" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="CONF_G2_DIVERGENCIAS" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="CONF_G5_MENSAL" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="CAD_FICHA" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="CAD_AUDITORIA" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="DICIONARIOS" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="FONTES" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="PROG_RESUMO_MENSAL" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="PROG_EVENTOS_DESVIO" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="REN_FC_ANUAL" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="REN_FC_MENSAL" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="REN_CORTE_ANUAL" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="REN_CORTE_MENSAL" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="REN_CORTE_RAZAO" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="REN_RECURSO_FAIXAS" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="REN_DESVIOS_PROGRAMACAO" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="CONF_G1_PARES" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="CONF_G1_MENSAL" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="CONF_G2_MENSAL" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="CONF_G2_DIVERGENCIAS" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="CONF_G5_MENSAL" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="CAD_FICHA" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="CAD_AUDITORIA" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="DICIONARIOS" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="FONTES" sheetId="27" state="visible" r:id="rId27"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -440,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -498,46 +501,58 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Fator de capacidade</t>
+          <t>Programação diária do ONS</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Fator de capacidade publicado pelo ONS de 16,7% de 22/08/2026 a 19/10/2026, no nível conjunto de usinas, em 1.416 horas.</t>
+          <t>Nas 1.296 horas com programação e geração verificada do conjunto Conj. Inocência 230 kV, geração verificada média de 69,6 MW e programada de 40,8 MW (desvio médio absoluto de 43,9 MW; correlação de 0,63); 4 horas com geração até 1 MW e programação acima de 5 MW.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Energia cortada</t>
+          <t>Fator de capacidade</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Energia cortada por restrição de operação de 1.127 MWh nas 814 semi-horas com a marca de restrição (16,3% da energia estimada nas semi-horas com a marca); diferença bruta entre a estimada e a verificada de 2.428 MWh em todas as semi-horas. Sem a estimativa do ONS (estimada 0 com a usina gerando) em 500 semi-horas, 385 delas com a marca de restrição, em que o corte não pôde ser calculado.</t>
+          <t>Fator de capacidade publicado pelo ONS de 16,7% de 22/08/2026 a 19/10/2026, no nível conjunto de usinas, em 1.416 horas.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Recurso × geração</t>
+          <t>Energia cortada</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Medição de irradiância marcada como inválida pelo ONS em 564 das 2.832 semi-horas (19,9%), fora das faixas.</t>
+          <t>Energia cortada por restrição de operação de 1.127 MWh nas 814 semi-horas com a marca de restrição (16,3% da energia estimada nas semi-horas com a marca); diferença bruta entre a estimada e a verificada de 2.428 MWh em todas as semi-horas. Sem a estimativa do ONS (estimada 0 com a usina gerando) em 500 semi-horas, 385 delas com a marca de restrição, em que o corte não pôde ser calculado.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>Recurso × geração</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Medição de irradiância marcada como inválida pelo ONS em 564 das 2.832 semi-horas (19,9%), fora das faixas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>Qualidade dos dados</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>Nenhuma hora sinalizada na base horária.</t>
         </is>
@@ -549,6 +564,219 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="27" customWidth="1" min="6" max="6"/>
+    <col width="27" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>mes</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>horas_comuns</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>geracao_media_mw</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>programada_media_mw</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>desvio_medio_mw</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>desvio_medio_absoluto_mw</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>horas_desvio_programacao</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B2" t="n">
+        <v>120</v>
+      </c>
+      <c r="C2" t="n">
+        <v>82.20726666666665</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>82.20726666666665</v>
+      </c>
+      <c r="F2" t="n">
+        <v>82.20726666666665</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B3" t="n">
+        <v>720</v>
+      </c>
+      <c r="C3" t="n">
+        <v>68.72983402777777</v>
+      </c>
+      <c r="D3" t="n">
+        <v>42.25694444444444</v>
+      </c>
+      <c r="E3" t="n">
+        <v>26.47288958333333</v>
+      </c>
+      <c r="F3" t="n">
+        <v>39.47373263888889</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B4" t="n">
+        <v>456</v>
+      </c>
+      <c r="C4" t="n">
+        <v>67.65447807017544</v>
+      </c>
+      <c r="D4" t="n">
+        <v>49.13925438596491</v>
+      </c>
+      <c r="E4" t="n">
+        <v>18.51522368421053</v>
+      </c>
+      <c r="F4" t="n">
+        <v>40.81308114035087</v>
+      </c>
+      <c r="G4" t="n">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>inicio</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>fim</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>duracao_h</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>programacao_media_mw</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n">
+        <v>46295.25</v>
+      </c>
+      <c r="B2" s="1" t="n">
+        <v>46295.25</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n">
+        <v>46304.66666666666</v>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>46304.70833333334</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="n">
+        <v>183.25</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n">
+        <v>46308.70833333334</v>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>46308.70833333334</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="n">
+        <v>67.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -651,7 +879,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -801,7 +1029,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -938,7 +1166,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1217,7 +1445,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1286,7 +1514,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1521,7 +1749,259 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>din_instante</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>geracao_programada_mw</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>geracao_mw</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>desvio_mw</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n">
+        <v>46267.58333333334</v>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" t="n">
+        <v>391.3095</v>
+      </c>
+      <c r="D2" t="n">
+        <v>391.3095</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n">
+        <v>46267.625</v>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" t="n">
+        <v>388.6385</v>
+      </c>
+      <c r="D3" t="n">
+        <v>388.6385</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n">
+        <v>46268.625</v>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" t="n">
+        <v>386.31</v>
+      </c>
+      <c r="D4" t="n">
+        <v>386.31</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="n">
+        <v>46267.33333333334</v>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" t="n">
+        <v>377.784</v>
+      </c>
+      <c r="D5" t="n">
+        <v>377.784</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="n">
+        <v>46267.41666666666</v>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" t="n">
+        <v>376.3165</v>
+      </c>
+      <c r="D6" t="n">
+        <v>376.3165</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="n">
+        <v>46267.45833333334</v>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" t="n">
+        <v>374.988</v>
+      </c>
+      <c r="D7" t="n">
+        <v>374.988</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>46262.58333333334</v>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" t="n">
+        <v>364.955</v>
+      </c>
+      <c r="D8" t="n">
+        <v>364.955</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
+        <v>46261.45833333334</v>
+      </c>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" t="n">
+        <v>352.705</v>
+      </c>
+      <c r="D9" t="n">
+        <v>352.705</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="n">
+        <v>46261.41666666666</v>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" t="n">
+        <v>350</v>
+      </c>
+      <c r="D10" t="n">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n">
+        <v>46262.625</v>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" t="n">
+        <v>350</v>
+      </c>
+      <c r="D11" t="n">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="n">
+        <v>46263.375</v>
+      </c>
+      <c r="B12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" t="n">
+        <v>348.073</v>
+      </c>
+      <c r="D12" t="n">
+        <v>348.073</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="n">
+        <v>46263.41666666666</v>
+      </c>
+      <c r="B13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" t="n">
+        <v>347.927</v>
+      </c>
+      <c r="D13" t="n">
+        <v>347.927</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="n">
+        <v>46261.5</v>
+      </c>
+      <c r="B14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" t="n">
+        <v>346.836</v>
+      </c>
+      <c r="D14" t="n">
+        <v>346.836</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="n">
+        <v>46261.375</v>
+      </c>
+      <c r="B15" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" t="n">
+        <v>344.0525</v>
+      </c>
+      <c r="D15" t="n">
+        <v>344.0525</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="n">
+        <v>46268.66666666666</v>
+      </c>
+      <c r="B16" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" t="n">
+        <v>338.408</v>
+      </c>
+      <c r="D16" t="n">
+        <v>338.408</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1728,7 +2208,105 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>lista</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>ordem</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>regra</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>secoes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Pontos de atenção</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>C16</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Energia cortada por restrição de operação de 1.127 MWh, 16,3% da energia estimada nas semi-horas com a marca de restrição</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>7. Energia cortada por restrição de operação (constrained-off)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>A verificar em campo</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>C17</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Medição de irradiância marcada como inválida pelo ONS em 564 das 2.832 semi-horas da usina (19,9%)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>8. Recurso × geração</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2199,7 +2777,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2349,7 +2927,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3434,105 +4012,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>lista</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>ordem</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>regra</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>texto</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>secoes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Pontos de atenção</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>C16</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Energia cortada por restrição de operação de 1.127 MWh, 16,3% da energia estimada nas semi-horas com a marca de restrição</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>7. Energia cortada por restrição de operação (constrained-off)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>A verificar em campo</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>C17</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Medição de irradiância marcada como inválida pelo ONS em 564 das 2.832 semi-horas da usina (19,9%)</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>8. Recurso × geração</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3682,7 +4162,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3859,7 +4339,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3964,7 +4444,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4832,13 +5312,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -5121,22 +5601,22 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>REN_FC_ANUAL</t>
+          <t>PROG_RESUMO_MENSAL</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Fator de capacidade (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; parâmetros do projeto (origem na tabela de parâmetros)</t>
+          <t>Programação diária (conjunto de usinas, MS4FINO), obtido em 20/10/2026; Geração por usina (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>geração conferida entre as fontes, duas a duas e no mesmo nível (G1): 4.248 de 4.248 horas coincidentes (100,0%) em 3 pares de fontes, detalhados na aba CONF_G1_PARES; programação diária conferida com o programado do Fator de capacidade (G5): 1.104 de 1.104 horas coincidentes (100,0%), 192 horas só numa das fontes</t>
+          <t>programação diária conferida com o programado do Fator de capacidade (G5): 1.104 de 1.104 horas coincidentes (100,0%), 192 horas só numa das fontes</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>geração</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -5148,22 +5628,22 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>REN_FC_MENSAL</t>
+          <t>PROG_EVENTOS_DESVIO</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Fator de capacidade (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; parâmetros do projeto (origem na tabela de parâmetros)</t>
+          <t>Programação diária (conjunto de usinas, MS4FINO), obtido em 20/10/2026; Geração por usina (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>geração conferida entre as fontes, duas a duas e no mesmo nível (G1): 4.248 de 4.248 horas coincidentes (100,0%) em 3 pares de fontes, detalhados na aba CONF_G1_PARES; programação diária conferida com o programado do Fator de capacidade (G5): 1.104 de 1.104 horas coincidentes (100,0%), 192 horas só numa das fontes</t>
+          <t>programação diária conferida com o programado do Fator de capacidade (G5): 1.104 de 1.104 horas coincidentes (100,0%), 192 horas só numa das fontes</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>geração</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -5175,22 +5655,22 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>REN_CORTE_ANUAL</t>
+          <t>REN_FC_ANUAL</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026</t>
+          <t>Fator de capacidade (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; parâmetros do projeto (origem na tabela de parâmetros)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>geração conferida entre as fontes, duas a duas e no mesmo nível (G1): 4.248 de 4.248 horas coincidentes (100,0%) em 3 pares de fontes, detalhados na aba CONF_G1_PARES; soma das usinas do conjunto (Restrição com detalhe) conferida com a Geração por usina do conjunto (G2): 1.105 de 1.296 horas coincidentes (85,3%), 191 divergências, listadas na aba CONF_G2_DIVERGENCIAS; 120 horas sem todas as usinas, fora da soma</t>
+          <t>geração conferida entre as fontes, duas a duas e no mesmo nível (G1): 4.248 de 4.248 horas coincidentes (100,0%) em 3 pares de fontes, detalhados na aba CONF_G1_PARES; programação diária conferida com o programado do Fator de capacidade (G5): 1.104 de 1.104 horas coincidentes (100,0%), 192 horas só numa das fontes</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>geração estimada e marca de restrição</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -5202,22 +5682,22 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>REN_CORTE_MENSAL</t>
+          <t>REN_FC_MENSAL</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Restrição com a razão (constrained-off) (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
+          <t>Fator de capacidade (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; parâmetros do projeto (origem na tabela de parâmetros)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>geração conferida entre as fontes, duas a duas e no mesmo nível (G1): 4.248 de 4.248 horas coincidentes (100,0%) em 3 pares de fontes, detalhados na aba CONF_G1_PARES</t>
+          <t>geração conferida entre as fontes, duas a duas e no mesmo nível (G1): 4.248 de 4.248 horas coincidentes (100,0%) em 3 pares de fontes, detalhados na aba CONF_G1_PARES; programação diária conferida com o programado do Fator de capacidade (G5): 1.104 de 1.104 horas coincidentes (100,0%), 192 horas só numa das fontes</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>geração estimada e marca de restrição</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -5229,17 +5709,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>REN_CORTE_RAZAO</t>
+          <t>REN_CORTE_ANUAL</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Restrição com a razão (constrained-off) (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
+          <t>Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>geração conferida entre as fontes, duas a duas e no mesmo nível (G1): 4.248 de 4.248 horas coincidentes (100,0%) em 3 pares de fontes, detalhados na aba CONF_G1_PARES</t>
+          <t>geração conferida entre as fontes, duas a duas e no mesmo nível (G1): 4.248 de 4.248 horas coincidentes (100,0%) em 3 pares de fontes, detalhados na aba CONF_G1_PARES; soma das usinas do conjunto (Restrição com detalhe) conferida com a Geração por usina do conjunto (G2): 1.105 de 1.296 horas coincidentes (85,3%), 191 divergências, listadas na aba CONF_G2_DIVERGENCIAS; 120 horas sem todas as usinas, fora da soma</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -5256,12 +5736,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>REN_RECURSO_FAIXAS</t>
+          <t>REN_CORTE_MENSAL</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026</t>
+          <t>Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Restrição com a razão (constrained-off) (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -5271,7 +5751,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>vento ou irradiância</t>
+          <t>geração estimada e marca de restrição</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -5283,12 +5763,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CONF_G1_PARES</t>
+          <t>REN_CORTE_RAZAO</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Geração por usina (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Fator de capacidade (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Restrição com a razão (constrained-off) (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
+          <t>Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Restrição com a razão (constrained-off) (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -5298,24 +5778,24 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>geração estimada e marca de restrição</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>não</t>
+          <t>sim</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CONF_G1_MENSAL</t>
+          <t>REN_RECURSO_FAIXAS</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Geração por usina (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Fator de capacidade (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Restrição com a razão (constrained-off) (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
+          <t>Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -5325,29 +5805,29 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>vento ou irradiância</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>não</t>
+          <t>sim</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CONF_G2_MENSAL</t>
+          <t>REN_DESVIOS_PROGRAMACAO</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Geração por usina (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
+          <t>Programação diária (conjunto de usinas, MS4FINO), obtido em 20/10/2026; Geração por usina (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>soma das usinas do conjunto (Restrição com detalhe) conferida com a Geração por usina do conjunto (G2): 1.105 de 1.296 horas coincidentes (85,3%), 191 divergências, listadas na aba CONF_G2_DIVERGENCIAS; 120 horas sem todas as usinas, fora da soma</t>
+          <t>programação diária conferida com o programado do Fator de capacidade (G5): 1.104 de 1.104 horas coincidentes (100,0%), 192 horas só numa das fontes</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -5364,17 +5844,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CONF_G2_DIVERGENCIAS</t>
+          <t>CONF_G1_PARES</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Geração por usina (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
+          <t>Geração por usina (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Fator de capacidade (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Restrição com a razão (constrained-off) (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>soma das usinas do conjunto (Restrição com detalhe) conferida com a Geração por usina do conjunto (G2): 1.105 de 1.296 horas coincidentes (85,3%), 191 divergências, listadas na aba CONF_G2_DIVERGENCIAS; 120 horas sem todas as usinas, fora da soma</t>
+          <t>geração conferida entre as fontes, duas a duas e no mesmo nível (G1): 4.248 de 4.248 horas coincidentes (100,0%) em 3 pares de fontes, detalhados na aba CONF_G1_PARES</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -5391,17 +5871,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CONF_G5_MENSAL</t>
+          <t>CONF_G1_MENSAL</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Programação diária (conjunto de usinas, MS4FINO), obtido em 20/10/2026; Fator de capacidade (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
+          <t>Geração por usina (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Fator de capacidade (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Restrição com a razão (constrained-off) (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>programação diária conferida com o programado do Fator de capacidade (G5): 1.104 de 1.104 horas coincidentes (100,0%), 192 horas só numa das fontes</t>
+          <t>geração conferida entre as fontes, duas a duas e no mesmo nível (G1): 4.248 de 4.248 horas coincidentes (100,0%) em 3 pares de fontes, detalhados na aba CONF_G1_PARES</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -5418,17 +5898,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CAD_FICHA</t>
+          <t>CONF_G2_MENSAL</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Modalidade das usinas (CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026</t>
+          <t>Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Geração por usina (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>potência autorizada e estado conferidos com os parâmetros do projeto: divergências (potência autorizada de 2,5 MW (projeto: 50 MW))</t>
+          <t>soma das usinas do conjunto (Restrição com detalhe) conferida com a Geração por usina do conjunto (G2): 1.105 de 1.296 horas coincidentes (85,3%), 191 divergências, listadas na aba CONF_G2_DIVERGENCIAS; 120 horas sem todas as usinas, fora da soma</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -5445,17 +5925,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CAD_AUDITORIA</t>
+          <t>CONF_G2_DIVERGENCIAS</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Modalidade das usinas (CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026</t>
+          <t>Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Geração por usina (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>soma das usinas do conjunto (Restrição com detalhe) conferida com a Geração por usina do conjunto (G2): 1.105 de 1.296 horas coincidentes (85,3%), 191 divergências, listadas na aba CONF_G2_DIVERGENCIAS; 120 horas sem todas as usinas, fora da soma</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -5472,25 +5952,106 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>CONF_G5_MENSAL</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Programação diária (conjunto de usinas, MS4FINO), obtido em 20/10/2026; Fator de capacidade (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>programação diária conferida com o programado do Fator de capacidade (G5): 1.104 de 1.104 horas coincidentes (100,0%), 192 horas só numa das fontes</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>CAD_FICHA</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Modalidade das usinas (CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>potência autorizada e estado conferidos com os parâmetros do projeto: divergências (potência autorizada de 2,5 MW (projeto: 50 MW))</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>CAD_AUDITORIA</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Modalidade das usinas (CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>DICIONARIOS</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>Programação diária (conjunto de usinas, MS4FINO), obtido em 20/10/2026; Geração por usina (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Modalidade das usinas (CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Composição dos conjuntos de usinas (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Capacidade de geração (CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Fator de capacidade (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Restrição com a razão (constrained-off) (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>não</t>
         </is>
@@ -6314,7 +6875,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -6376,7 +6937,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Programação diária × geração verificada</t>
+          <t>Conferência da geração entre fontes</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -6386,31 +6947,31 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>sem horas com a programação e a geração verificada no mesmo nível</t>
+          <t>seção ainda não gerada pelo pipeline; os resultados da G1, da G2 e da G5, quando aplicáveis, estão nas legendas de fonte das seções de eólica e solar e nas abas CONF_G1, CONF_G2 e CONF_G5 da planilha</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Conferência da geração entre fontes</t>
+          <t>C18</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>secao</t>
+          <t>regra</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>seção ainda não gerada pelo pipeline; os resultados da G1, da G2 e da G5, quando aplicáveis, estão nas legendas de fonte das seções de eólica e solar e nas abas CONF_G1, CONF_G2 e CONF_G5 da planilha</t>
+          <t>sem o Fator de capacidade no nível da usina</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C18</t>
+          <t>C19</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -6419,23 +6980,6 @@
         </is>
       </c>
       <c r="C6" t="inlineStr">
-        <is>
-          <t>sem o Fator de capacidade no nível da usina</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>C19</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>regra</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
         <is>
           <t>sem a Programação diária no nível da usina</t>
         </is>

</xml_diff>